<commit_message>
Update with leads edit/delete and manual client entry
</commit_message>
<xml_diff>
--- a/backend/data/sip_advisor_enriched_preview.xlsx
+++ b/backend/data/sip_advisor_enriched_preview.xlsx
@@ -599,11 +599,11 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>19-07-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="O2" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -623,7 +623,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>19-06-2026</t>
+          <t>19-07-2026</t>
         </is>
       </c>
       <c r="U2" t="b">
@@ -694,31 +694,31 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>16-08-2026</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>19</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S3" t="b">
+        <v>0</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>16-07-2026</t>
-        </is>
-      </c>
-      <c r="O3" t="n">
-        <v>11</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S3" t="b">
-        <v>0</v>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>16-06-2026</t>
         </is>
       </c>
       <c r="U3" t="b">
@@ -789,11 +789,11 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>28-07-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="O4" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
@@ -813,7 +813,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>28-06-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="U4" t="b">
@@ -884,11 +884,11 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>28-07-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="O5" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
@@ -908,7 +908,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>28-06-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="U5" t="b">
@@ -979,31 +979,31 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S6" t="b">
+        <v>0</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
           <t>12-07-2026</t>
-        </is>
-      </c>
-      <c r="O6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S6" t="b">
-        <v>0</v>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>12-06-2026</t>
         </is>
       </c>
       <c r="U6" t="b">
@@ -1074,31 +1074,31 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>17-08-2026</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>20</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S7" t="b">
+        <v>0</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
           <t>17-07-2026</t>
-        </is>
-      </c>
-      <c r="O7" t="n">
-        <v>12</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S7" t="b">
-        <v>0</v>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>17-06-2026</t>
         </is>
       </c>
       <c r="U7" t="b">
@@ -1169,31 +1169,31 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
+          <t>14-08-2026</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>17</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S8" t="b">
+        <v>0</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
           <t>14-07-2026</t>
-        </is>
-      </c>
-      <c r="O8" t="n">
-        <v>9</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S8" t="b">
-        <v>0</v>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>14-06-2026</t>
         </is>
       </c>
       <c r="U8" t="b">
@@ -1268,7 +1268,7 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -1359,11 +1359,11 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="O10" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="P10" t="n">
         <v>1</v>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="U10" t="b">
@@ -1454,11 +1454,11 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>19-07-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="O11" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>19-06-2026</t>
+          <t>19-07-2026</t>
         </is>
       </c>
       <c r="U11" t="b">
@@ -1549,31 +1549,31 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
+          <t>13-08-2026</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>16</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S12" t="b">
+        <v>0</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
           <t>13-07-2026</t>
-        </is>
-      </c>
-      <c r="O12" t="n">
-        <v>8</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S12" t="b">
-        <v>0</v>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>13-06-2026</t>
         </is>
       </c>
       <c r="U12" t="b">
@@ -1644,11 +1644,11 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="O13" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="P13" t="n">
         <v>1</v>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>11-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="U13" t="b">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>15-07-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="O14" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="P14" t="n">
         <v>1</v>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>15-07-2026</t>
         </is>
       </c>
       <c r="U14" t="b">
@@ -1834,31 +1834,31 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
+          <t>15-08-2026</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>18</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S15" t="b">
+        <v>0</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
           <t>15-07-2026</t>
-        </is>
-      </c>
-      <c r="O15" t="n">
-        <v>10</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S15" t="b">
-        <v>0</v>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>15-06-2026</t>
         </is>
       </c>
       <c r="U15" t="b">
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="P16" t="n">
         <v>3</v>
@@ -2024,31 +2024,31 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>15</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S17" t="b">
+        <v>0</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
           <t>12-07-2026</t>
-        </is>
-      </c>
-      <c r="O17" t="n">
-        <v>7</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S17" t="b">
-        <v>0</v>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>12-06-2026</t>
         </is>
       </c>
       <c r="U17" t="b">
@@ -2119,11 +2119,11 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>12-07-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="O18" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -2143,7 +2143,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>12-07-2026</t>
         </is>
       </c>
       <c r="U18" t="b">
@@ -2214,11 +2214,11 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>28-07-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="O19" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="P19" t="n">
         <v>1</v>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>28-06-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="U19" t="b">
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="P20" t="n">
         <v>1</v>
@@ -2408,7 +2408,7 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
@@ -2503,7 +2503,7 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
@@ -2527,7 +2527,7 @@
         </is>
       </c>
       <c r="U22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2598,7 +2598,7 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="P23" t="n">
         <v>2</v>
@@ -2622,7 +2622,7 @@
         </is>
       </c>
       <c r="U23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -2689,11 +2689,11 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>28-07-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="O24" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>28-06-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="U24" t="b">
@@ -2784,31 +2784,31 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
+          <t>28-08-2026</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>31</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S25" t="b">
+        <v>0</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
           <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="O25" t="n">
-        <v>23</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S25" t="b">
-        <v>0</v>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>28-06-2026</t>
         </is>
       </c>
       <c r="U25" t="b">
@@ -2879,11 +2879,11 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>12-07-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="O26" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="P26" t="n">
         <v>1</v>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>12-07-2026</t>
         </is>
       </c>
       <c r="U26" t="b">
@@ -2974,11 +2974,11 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>21-07-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="O27" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="P27" t="n">
         <v>2</v>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>21-07-2026</t>
         </is>
       </c>
       <c r="U27" t="b">
@@ -3069,31 +3069,31 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>14</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S28" t="b">
+        <v>0</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
           <t>11-07-2026</t>
-        </is>
-      </c>
-      <c r="O28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S28" t="b">
-        <v>0</v>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>11-06-2026</t>
         </is>
       </c>
       <c r="U28" t="b">
@@ -3168,7 +3168,7 @@
         </is>
       </c>
       <c r="O29" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="P29" t="n">
         <v>1</v>
@@ -3259,35 +3259,35 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
+          <t>07-08-2026</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>10</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S30" t="b">
+        <v>0</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
           <t>07-07-2026</t>
         </is>
       </c>
-      <c r="O30" t="n">
-        <v>2</v>
-      </c>
-      <c r="P30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S30" t="b">
-        <v>0</v>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>07-06-2026</t>
-        </is>
-      </c>
       <c r="U30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="O31" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="P31" t="n">
         <v>0</v>
@@ -3449,11 +3449,11 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>19-07-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="O32" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="P32" t="n">
         <v>1</v>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>19-06-2026</t>
+          <t>19-07-2026</t>
         </is>
       </c>
       <c r="U32" t="b">
@@ -3544,11 +3544,11 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>19-07-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="O33" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="P33" t="n">
         <v>1</v>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>19-06-2026</t>
+          <t>19-07-2026</t>
         </is>
       </c>
       <c r="U33" t="b">
@@ -3643,7 +3643,7 @@
         </is>
       </c>
       <c r="O34" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="U34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -3734,31 +3734,31 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
+          <t>13-08-2026</t>
+        </is>
+      </c>
+      <c r="O35" t="n">
+        <v>16</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S35" t="b">
+        <v>0</v>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
           <t>13-07-2026</t>
-        </is>
-      </c>
-      <c r="O35" t="n">
-        <v>8</v>
-      </c>
-      <c r="P35" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S35" t="b">
-        <v>0</v>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>13-06-2026</t>
         </is>
       </c>
       <c r="U35" t="b">
@@ -3833,7 +3833,7 @@
         </is>
       </c>
       <c r="O36" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="P36" t="n">
         <v>0</v>
@@ -3857,7 +3857,7 @@
         </is>
       </c>
       <c r="U36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -3924,11 +3924,11 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>20-07-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="O37" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="P37" t="n">
         <v>0</v>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>20-06-2026</t>
+          <t>20-07-2026</t>
         </is>
       </c>
       <c r="U37" t="b">
@@ -4019,11 +4019,11 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="O38" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="P38" t="n">
         <v>2</v>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>10-07-2026</t>
         </is>
       </c>
       <c r="U38" t="b">
@@ -4114,11 +4114,11 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>17-07-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="O39" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P39" t="n">
         <v>0</v>
@@ -4138,7 +4138,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>17-06-2026</t>
+          <t>17-07-2026</t>
         </is>
       </c>
       <c r="U39" t="b">
@@ -4209,11 +4209,11 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="O40" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="P40" t="n">
         <v>2</v>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>11-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="U40" t="b">
@@ -4304,31 +4304,31 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
+          <t>23-08-2026</t>
+        </is>
+      </c>
+      <c r="O41" t="n">
+        <v>26</v>
+      </c>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S41" t="b">
+        <v>0</v>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
           <t>23-07-2026</t>
-        </is>
-      </c>
-      <c r="O41" t="n">
-        <v>18</v>
-      </c>
-      <c r="P41" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S41" t="b">
-        <v>0</v>
-      </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t>23-06-2026</t>
         </is>
       </c>
       <c r="U41" t="b">
@@ -4399,11 +4399,11 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>27-07-2026</t>
+          <t>27-08-2026</t>
         </is>
       </c>
       <c r="O42" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="P42" t="n">
         <v>3</v>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>27-06-2026</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="U42" t="b">
@@ -4494,11 +4494,11 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>12-07-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="O43" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="P43" t="n">
         <v>2</v>
@@ -4518,7 +4518,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>12-07-2026</t>
         </is>
       </c>
       <c r="U43" t="b">
@@ -4589,31 +4589,31 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
+          <t>14-08-2026</t>
+        </is>
+      </c>
+      <c r="O44" t="n">
+        <v>17</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S44" t="b">
+        <v>0</v>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
           <t>14-07-2026</t>
-        </is>
-      </c>
-      <c r="O44" t="n">
-        <v>9</v>
-      </c>
-      <c r="P44" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S44" t="b">
-        <v>0</v>
-      </c>
-      <c r="T44" t="inlineStr">
-        <is>
-          <t>14-06-2026</t>
         </is>
       </c>
       <c r="U44" t="b">
@@ -4684,31 +4684,31 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
+          <t>10-08-2026</t>
+        </is>
+      </c>
+      <c r="O45" t="n">
+        <v>13</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S45" t="b">
+        <v>0</v>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
           <t>10-07-2026</t>
-        </is>
-      </c>
-      <c r="O45" t="n">
-        <v>5</v>
-      </c>
-      <c r="P45" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S45" t="b">
-        <v>0</v>
-      </c>
-      <c r="T45" t="inlineStr">
-        <is>
-          <t>10-06-2026</t>
         </is>
       </c>
       <c r="U45" t="b">
@@ -4779,11 +4779,11 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>27-07-2026</t>
+          <t>27-08-2026</t>
         </is>
       </c>
       <c r="O46" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="P46" t="n">
         <v>0</v>
@@ -4803,7 +4803,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>27-06-2026</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="U46" t="b">
@@ -4874,31 +4874,31 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="O47" t="n">
+        <v>14</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S47" t="b">
+        <v>0</v>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
           <t>11-07-2026</t>
-        </is>
-      </c>
-      <c r="O47" t="n">
-        <v>6</v>
-      </c>
-      <c r="P47" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S47" t="b">
-        <v>0</v>
-      </c>
-      <c r="T47" t="inlineStr">
-        <is>
-          <t>11-06-2026</t>
         </is>
       </c>
       <c r="U47" t="b">
@@ -4973,7 +4973,7 @@
         </is>
       </c>
       <c r="O48" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="P48" t="n">
         <v>0</v>
@@ -4997,7 +4997,7 @@
         </is>
       </c>
       <c r="U48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -5064,11 +5064,11 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>08-08-2026</t>
         </is>
       </c>
       <c r="O49" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="P49" t="n">
         <v>1</v>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="U49" t="b">
@@ -5159,11 +5159,11 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>19-07-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="O50" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="P50" t="n">
         <v>2</v>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>19-06-2026</t>
+          <t>19-07-2026</t>
         </is>
       </c>
       <c r="U50" t="b">
@@ -5254,31 +5254,31 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="O51" t="n">
+        <v>14</v>
+      </c>
+      <c r="P51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S51" t="b">
+        <v>0</v>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
           <t>11-07-2026</t>
-        </is>
-      </c>
-      <c r="O51" t="n">
-        <v>6</v>
-      </c>
-      <c r="P51" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S51" t="b">
-        <v>0</v>
-      </c>
-      <c r="T51" t="inlineStr">
-        <is>
-          <t>11-06-2026</t>
         </is>
       </c>
       <c r="U51" t="b">
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="O52" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="P52" t="n">
         <v>0</v>
@@ -5377,7 +5377,7 @@
         </is>
       </c>
       <c r="U52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -5448,7 +5448,7 @@
         </is>
       </c>
       <c r="O53" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="P53" t="n">
         <v>1</v>
@@ -5472,7 +5472,7 @@
         </is>
       </c>
       <c r="U53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -5539,31 +5539,31 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
+          <t>17-08-2026</t>
+        </is>
+      </c>
+      <c r="O54" t="n">
+        <v>20</v>
+      </c>
+      <c r="P54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S54" t="b">
+        <v>0</v>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
           <t>17-07-2026</t>
-        </is>
-      </c>
-      <c r="O54" t="n">
-        <v>12</v>
-      </c>
-      <c r="P54" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S54" t="b">
-        <v>0</v>
-      </c>
-      <c r="T54" t="inlineStr">
-        <is>
-          <t>17-06-2026</t>
         </is>
       </c>
       <c r="U54" t="b">
@@ -5634,11 +5634,11 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>20-07-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="O55" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="P55" t="n">
         <v>1</v>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>20-06-2026</t>
+          <t>20-07-2026</t>
         </is>
       </c>
       <c r="U55" t="b">
@@ -5733,7 +5733,7 @@
         </is>
       </c>
       <c r="O56" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="P56" t="n">
         <v>0</v>
@@ -5828,7 +5828,7 @@
         </is>
       </c>
       <c r="O57" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="P57" t="n">
         <v>0</v>
@@ -5919,11 +5919,11 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="O58" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="P58" t="n">
         <v>0</v>
@@ -5943,7 +5943,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>10-07-2026</t>
         </is>
       </c>
       <c r="U58" t="b">
@@ -6014,11 +6014,11 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>22-07-2026</t>
+          <t>22-08-2026</t>
         </is>
       </c>
       <c r="O59" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="P59" t="n">
         <v>2</v>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>22-06-2026</t>
+          <t>22-07-2026</t>
         </is>
       </c>
       <c r="U59" t="b">
@@ -6109,11 +6109,11 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>06-07-2026</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="O60" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="P60" t="n">
         <v>1</v>
@@ -6133,11 +6133,11 @@
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>06-06-2026</t>
+          <t>06-07-2026</t>
         </is>
       </c>
       <c r="U60" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -6204,11 +6204,11 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>19-07-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="O61" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="P61" t="n">
         <v>1</v>
@@ -6228,7 +6228,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>19-06-2026</t>
+          <t>19-07-2026</t>
         </is>
       </c>
       <c r="U61" t="b">
@@ -6299,11 +6299,11 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>24-08-2026</t>
         </is>
       </c>
       <c r="O62" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="P62" t="n">
         <v>1</v>
@@ -6323,7 +6323,7 @@
       </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="U62" t="b">
@@ -6394,11 +6394,11 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>08-08-2026</t>
         </is>
       </c>
       <c r="O63" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="P63" t="n">
         <v>1</v>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="U63" t="b">
@@ -6489,31 +6489,31 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
+          <t>13-08-2026</t>
+        </is>
+      </c>
+      <c r="O64" t="n">
+        <v>16</v>
+      </c>
+      <c r="P64" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S64" t="b">
+        <v>0</v>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
           <t>13-07-2026</t>
-        </is>
-      </c>
-      <c r="O64" t="n">
-        <v>8</v>
-      </c>
-      <c r="P64" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q64" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R64" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S64" t="b">
-        <v>0</v>
-      </c>
-      <c r="T64" t="inlineStr">
-        <is>
-          <t>13-06-2026</t>
         </is>
       </c>
       <c r="U64" t="b">
@@ -6584,31 +6584,31 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
+          <t>10-08-2026</t>
+        </is>
+      </c>
+      <c r="O65" t="n">
+        <v>13</v>
+      </c>
+      <c r="P65" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S65" t="b">
+        <v>0</v>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
           <t>10-07-2026</t>
-        </is>
-      </c>
-      <c r="O65" t="n">
-        <v>5</v>
-      </c>
-      <c r="P65" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q65" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S65" t="b">
-        <v>0</v>
-      </c>
-      <c r="T65" t="inlineStr">
-        <is>
-          <t>10-06-2026</t>
         </is>
       </c>
       <c r="U65" t="b">
@@ -6679,11 +6679,11 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>23-08-2026</t>
         </is>
       </c>
       <c r="O66" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="P66" t="n">
         <v>2</v>
@@ -6703,7 +6703,7 @@
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>23-06-2026</t>
+          <t>23-07-2026</t>
         </is>
       </c>
       <c r="U66" t="b">
@@ -6774,11 +6774,11 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>17-07-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="O67" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P67" t="n">
         <v>4</v>
@@ -6798,7 +6798,7 @@
       </c>
       <c r="T67" t="inlineStr">
         <is>
-          <t>17-06-2026</t>
+          <t>17-07-2026</t>
         </is>
       </c>
       <c r="U67" t="b">
@@ -6873,7 +6873,7 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="P68" t="n">
         <v>0</v>
@@ -6968,7 +6968,7 @@
         </is>
       </c>
       <c r="O69" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="P69" t="n">
         <v>0</v>
@@ -7059,11 +7059,11 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>08-08-2026</t>
         </is>
       </c>
       <c r="O70" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="P70" t="n">
         <v>2</v>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="T70" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="U70" t="b">
@@ -7158,7 +7158,7 @@
         </is>
       </c>
       <c r="O71" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="P71" t="n">
         <v>1</v>
@@ -7182,7 +7182,7 @@
         </is>
       </c>
       <c r="U71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -7253,7 +7253,7 @@
         </is>
       </c>
       <c r="O72" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="P72" t="n">
         <v>0</v>
@@ -7348,7 +7348,7 @@
         </is>
       </c>
       <c r="O73" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="P73" t="n">
         <v>0</v>
@@ -7372,7 +7372,7 @@
         </is>
       </c>
       <c r="U73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -7439,11 +7439,11 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>14-07-2026</t>
+          <t>14-08-2026</t>
         </is>
       </c>
       <c r="O74" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="P74" t="n">
         <v>3</v>
@@ -7463,7 +7463,7 @@
       </c>
       <c r="T74" t="inlineStr">
         <is>
-          <t>14-06-2026</t>
+          <t>14-07-2026</t>
         </is>
       </c>
       <c r="U74" t="b">
@@ -7534,31 +7534,31 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
+          <t>25-08-2026</t>
+        </is>
+      </c>
+      <c r="O75" t="n">
+        <v>28</v>
+      </c>
+      <c r="P75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S75" t="b">
+        <v>0</v>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
           <t>25-07-2026</t>
-        </is>
-      </c>
-      <c r="O75" t="n">
-        <v>20</v>
-      </c>
-      <c r="P75" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q75" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S75" t="b">
-        <v>0</v>
-      </c>
-      <c r="T75" t="inlineStr">
-        <is>
-          <t>25-06-2026</t>
         </is>
       </c>
       <c r="U75" t="b">
@@ -7629,11 +7629,11 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>23-08-2026</t>
         </is>
       </c>
       <c r="O76" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="P76" t="n">
         <v>3</v>
@@ -7653,7 +7653,7 @@
       </c>
       <c r="T76" t="inlineStr">
         <is>
-          <t>23-06-2026</t>
+          <t>23-07-2026</t>
         </is>
       </c>
       <c r="U76" t="b">
@@ -7724,31 +7724,31 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
+          <t>22-08-2026</t>
+        </is>
+      </c>
+      <c r="O77" t="n">
+        <v>25</v>
+      </c>
+      <c r="P77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S77" t="b">
+        <v>0</v>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
           <t>22-07-2026</t>
-        </is>
-      </c>
-      <c r="O77" t="n">
-        <v>17</v>
-      </c>
-      <c r="P77" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q77" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R77" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S77" t="b">
-        <v>0</v>
-      </c>
-      <c r="T77" t="inlineStr">
-        <is>
-          <t>22-06-2026</t>
         </is>
       </c>
       <c r="U77" t="b">
@@ -7819,11 +7819,11 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>08-08-2026</t>
         </is>
       </c>
       <c r="O78" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="P78" t="n">
         <v>2</v>
@@ -7843,7 +7843,7 @@
       </c>
       <c r="T78" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="U78" t="b">
@@ -7914,31 +7914,31 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
+          <t>10-08-2026</t>
+        </is>
+      </c>
+      <c r="O79" t="n">
+        <v>13</v>
+      </c>
+      <c r="P79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S79" t="b">
+        <v>0</v>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
           <t>10-07-2026</t>
-        </is>
-      </c>
-      <c r="O79" t="n">
-        <v>5</v>
-      </c>
-      <c r="P79" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q79" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R79" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S79" t="b">
-        <v>0</v>
-      </c>
-      <c r="T79" t="inlineStr">
-        <is>
-          <t>10-06-2026</t>
         </is>
       </c>
       <c r="U79" t="b">
@@ -8009,11 +8009,11 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>26-07-2026</t>
+          <t>26-08-2026</t>
         </is>
       </c>
       <c r="O80" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="P80" t="n">
         <v>2</v>
@@ -8033,7 +8033,7 @@
       </c>
       <c r="T80" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>26-07-2026</t>
         </is>
       </c>
       <c r="U80" t="b">
@@ -8104,11 +8104,11 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>25-07-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
       <c r="O81" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="P81" t="n">
         <v>1</v>
@@ -8128,7 +8128,7 @@
       </c>
       <c r="T81" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>25-07-2026</t>
         </is>
       </c>
       <c r="U81" t="b">
@@ -8203,7 +8203,7 @@
         </is>
       </c>
       <c r="O82" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="P82" t="n">
         <v>1</v>
@@ -8298,7 +8298,7 @@
         </is>
       </c>
       <c r="O83" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="P83" t="n">
         <v>0</v>
@@ -8393,7 +8393,7 @@
         </is>
       </c>
       <c r="O84" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="P84" t="n">
         <v>2</v>
@@ -8484,11 +8484,11 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="O85" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="P85" t="n">
         <v>4</v>
@@ -8508,7 +8508,7 @@
       </c>
       <c r="T85" t="inlineStr">
         <is>
-          <t>11-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="U85" t="b">
@@ -8579,11 +8579,11 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="O86" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="P86" t="n">
         <v>1</v>
@@ -8603,7 +8603,7 @@
       </c>
       <c r="T86" t="inlineStr">
         <is>
-          <t>11-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="U86" t="b">
@@ -8674,11 +8674,11 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>14-07-2026</t>
+          <t>14-08-2026</t>
         </is>
       </c>
       <c r="O87" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="P87" t="n">
         <v>4</v>
@@ -8698,7 +8698,7 @@
       </c>
       <c r="T87" t="inlineStr">
         <is>
-          <t>14-06-2026</t>
+          <t>14-07-2026</t>
         </is>
       </c>
       <c r="U87" t="b">
@@ -8769,31 +8769,31 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
+          <t>28-08-2026</t>
+        </is>
+      </c>
+      <c r="O88" t="n">
+        <v>31</v>
+      </c>
+      <c r="P88" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S88" t="b">
+        <v>0</v>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
           <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="O88" t="n">
-        <v>23</v>
-      </c>
-      <c r="P88" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q88" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R88" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S88" t="b">
-        <v>0</v>
-      </c>
-      <c r="T88" t="inlineStr">
-        <is>
-          <t>28-06-2026</t>
         </is>
       </c>
       <c r="U88" t="b">
@@ -8864,11 +8864,11 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="O89" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="P89" t="n">
         <v>0</v>
@@ -8888,7 +8888,7 @@
       </c>
       <c r="T89" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>10-07-2026</t>
         </is>
       </c>
       <c r="U89" t="b">
@@ -8959,31 +8959,31 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="O90" t="n">
+        <v>15</v>
+      </c>
+      <c r="P90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S90" t="b">
+        <v>0</v>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
           <t>12-07-2026</t>
-        </is>
-      </c>
-      <c r="O90" t="n">
-        <v>7</v>
-      </c>
-      <c r="P90" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q90" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R90" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S90" t="b">
-        <v>0</v>
-      </c>
-      <c r="T90" t="inlineStr">
-        <is>
-          <t>12-06-2026</t>
         </is>
       </c>
       <c r="U90" t="b">
@@ -9058,7 +9058,7 @@
         </is>
       </c>
       <c r="O91" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="P91" t="n">
         <v>0</v>
@@ -9082,7 +9082,7 @@
         </is>
       </c>
       <c r="U91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -9149,11 +9149,11 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>08-08-2026</t>
         </is>
       </c>
       <c r="O92" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="P92" t="n">
         <v>0</v>
@@ -9173,7 +9173,7 @@
       </c>
       <c r="T92" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="U92" t="b">
@@ -9244,11 +9244,11 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>13-07-2026</t>
+          <t>13-08-2026</t>
         </is>
       </c>
       <c r="O93" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="P93" t="n">
         <v>0</v>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="T93" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>13-07-2026</t>
         </is>
       </c>
       <c r="U93" t="b">
@@ -9339,11 +9339,11 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>21-07-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="O94" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="P94" t="n">
         <v>1</v>
@@ -9363,7 +9363,7 @@
       </c>
       <c r="T94" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>21-07-2026</t>
         </is>
       </c>
       <c r="U94" t="b">
@@ -9434,31 +9434,31 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
+          <t>28-08-2026</t>
+        </is>
+      </c>
+      <c r="O95" t="n">
+        <v>31</v>
+      </c>
+      <c r="P95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S95" t="b">
+        <v>0</v>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
           <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="O95" t="n">
-        <v>23</v>
-      </c>
-      <c r="P95" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q95" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R95" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S95" t="b">
-        <v>0</v>
-      </c>
-      <c r="T95" t="inlineStr">
-        <is>
-          <t>28-06-2026</t>
         </is>
       </c>
       <c r="U95" t="b">
@@ -9529,11 +9529,11 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>08-08-2026</t>
         </is>
       </c>
       <c r="O96" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="P96" t="n">
         <v>2</v>
@@ -9553,7 +9553,7 @@
       </c>
       <c r="T96" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="U96" t="b">
@@ -9624,31 +9624,31 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
+          <t>22-08-2026</t>
+        </is>
+      </c>
+      <c r="O97" t="n">
+        <v>25</v>
+      </c>
+      <c r="P97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S97" t="b">
+        <v>0</v>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
           <t>22-07-2026</t>
-        </is>
-      </c>
-      <c r="O97" t="n">
-        <v>17</v>
-      </c>
-      <c r="P97" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q97" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R97" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S97" t="b">
-        <v>0</v>
-      </c>
-      <c r="T97" t="inlineStr">
-        <is>
-          <t>22-06-2026</t>
         </is>
       </c>
       <c r="U97" t="b">
@@ -9719,11 +9719,11 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="O98" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="P98" t="n">
         <v>1</v>
@@ -9743,7 +9743,7 @@
       </c>
       <c r="T98" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="U98" t="b">
@@ -9814,31 +9814,31 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
+          <t>24-08-2026</t>
+        </is>
+      </c>
+      <c r="O99" t="n">
+        <v>27</v>
+      </c>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S99" t="b">
+        <v>0</v>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
           <t>24-07-2026</t>
-        </is>
-      </c>
-      <c r="O99" t="n">
-        <v>19</v>
-      </c>
-      <c r="P99" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q99" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="R99" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="S99" t="b">
-        <v>0</v>
-      </c>
-      <c r="T99" t="inlineStr">
-        <is>
-          <t>24-06-2026</t>
         </is>
       </c>
       <c r="U99" t="b">
@@ -9909,11 +9909,11 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>20-07-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="O100" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="P100" t="n">
         <v>0</v>
@@ -9933,7 +9933,7 @@
       </c>
       <c r="T100" t="inlineStr">
         <is>
-          <t>20-06-2026</t>
+          <t>20-07-2026</t>
         </is>
       </c>
       <c r="U100" t="b">
@@ -10004,11 +10004,11 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>23-08-2026</t>
         </is>
       </c>
       <c r="O101" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="P101" t="n">
         <v>1</v>
@@ -10028,7 +10028,7 @@
       </c>
       <c r="T101" t="inlineStr">
         <is>
-          <t>23-06-2026</t>
+          <t>23-07-2026</t>
         </is>
       </c>
       <c r="U101" t="b">

</xml_diff>

<commit_message>
Add clear-dataset option to remove demo data before review
</commit_message>
<xml_diff>
--- a/backend/data/sip_advisor_enriched_preview.xlsx
+++ b/backend/data/sip_advisor_enriched_preview.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1521" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1521" uniqueCount="752">
   <si>
     <t>sr_no</t>
   </si>
@@ -2101,19 +2101,121 @@
     <t>14-08-2026</t>
   </si>
   <si>
+    <t>02-09-2026</t>
+  </si>
+  <si>
+    <t>18-08-2026</t>
+  </si>
+  <si>
+    <t>13-08-2026</t>
+  </si>
+  <si>
+    <t>11-08-2026</t>
+  </si>
+  <si>
+    <t>15-08-2026</t>
+  </si>
+  <si>
+    <t>05-09-2026</t>
+  </si>
+  <si>
+    <t>04-09-2026</t>
+  </si>
+  <si>
+    <t>29-08-2026</t>
+  </si>
+  <si>
+    <t>21-08-2026</t>
+  </si>
+  <si>
+    <t>07-08-2026</t>
+  </si>
+  <si>
+    <t>30-08-2026</t>
+  </si>
+  <si>
+    <t>20-08-2026</t>
+  </si>
+  <si>
+    <t>10-08-2026</t>
+  </si>
+  <si>
+    <t>23-08-2026</t>
+  </si>
+  <si>
+    <t>27-08-2026</t>
+  </si>
+  <si>
+    <t>08-08-2026</t>
+  </si>
+  <si>
+    <t>22-08-2026</t>
+  </si>
+  <si>
+    <t>06-08-2026</t>
+  </si>
+  <si>
+    <t>24-08-2026</t>
+  </si>
+  <si>
+    <t>25-08-2026</t>
+  </si>
+  <si>
+    <t>26-08-2026</t>
+  </si>
+  <si>
+    <t>31-08-2026</t>
+  </si>
+  <si>
+    <t>03-09-2026</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Missed</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>19-07-2026</t>
+  </si>
+  <si>
+    <t>16-07-2026</t>
+  </si>
+  <si>
+    <t>28-07-2026</t>
+  </si>
+  <si>
+    <t>12-07-2026</t>
+  </si>
+  <si>
+    <t>17-07-2026</t>
+  </si>
+  <si>
+    <t>14-07-2026</t>
+  </si>
+  <si>
     <t>02-08-2026</t>
   </si>
   <si>
-    <t>18-08-2026</t>
-  </si>
-  <si>
-    <t>13-08-2026</t>
-  </si>
-  <si>
-    <t>11-08-2026</t>
-  </si>
-  <si>
-    <t>15-08-2026</t>
+    <t>18-07-2026</t>
+  </si>
+  <si>
+    <t>13-07-2026</t>
+  </si>
+  <si>
+    <t>11-07-2026</t>
+  </si>
+  <si>
+    <t>15-07-2026</t>
   </si>
   <si>
     <t>05-08-2026</t>
@@ -2122,151 +2224,52 @@
     <t>04-08-2026</t>
   </si>
   <si>
-    <t>29-08-2026</t>
-  </si>
-  <si>
-    <t>21-08-2026</t>
-  </si>
-  <si>
-    <t>07-08-2026</t>
+    <t>29-07-2026</t>
+  </si>
+  <si>
+    <t>21-07-2026</t>
+  </si>
+  <si>
+    <t>07-07-2026</t>
   </si>
   <si>
     <t>30-07-2026</t>
   </si>
   <si>
-    <t>20-08-2026</t>
-  </si>
-  <si>
-    <t>10-08-2026</t>
-  </si>
-  <si>
-    <t>23-08-2026</t>
-  </si>
-  <si>
-    <t>27-08-2026</t>
-  </si>
-  <si>
-    <t>08-08-2026</t>
-  </si>
-  <si>
-    <t>22-08-2026</t>
-  </si>
-  <si>
-    <t>06-08-2026</t>
-  </si>
-  <si>
-    <t>24-08-2026</t>
-  </si>
-  <si>
-    <t>25-08-2026</t>
-  </si>
-  <si>
-    <t>26-08-2026</t>
+    <t>20-07-2026</t>
+  </si>
+  <si>
+    <t>10-07-2026</t>
+  </si>
+  <si>
+    <t>23-07-2026</t>
+  </si>
+  <si>
+    <t>27-07-2026</t>
+  </si>
+  <si>
+    <t>08-07-2026</t>
+  </si>
+  <si>
+    <t>22-07-2026</t>
+  </si>
+  <si>
+    <t>06-07-2026</t>
+  </si>
+  <si>
+    <t>24-07-2026</t>
+  </si>
+  <si>
+    <t>25-07-2026</t>
+  </si>
+  <si>
+    <t>26-07-2026</t>
   </si>
   <si>
     <t>31-07-2026</t>
   </si>
   <si>
     <t>03-08-2026</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Missed</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>19-07-2026</t>
-  </si>
-  <si>
-    <t>16-07-2026</t>
-  </si>
-  <si>
-    <t>28-07-2026</t>
-  </si>
-  <si>
-    <t>12-07-2026</t>
-  </si>
-  <si>
-    <t>17-07-2026</t>
-  </si>
-  <si>
-    <t>14-07-2026</t>
-  </si>
-  <si>
-    <t>02-07-2026</t>
-  </si>
-  <si>
-    <t>18-07-2026</t>
-  </si>
-  <si>
-    <t>13-07-2026</t>
-  </si>
-  <si>
-    <t>11-07-2026</t>
-  </si>
-  <si>
-    <t>15-07-2026</t>
-  </si>
-  <si>
-    <t>05-07-2026</t>
-  </si>
-  <si>
-    <t>04-07-2026</t>
-  </si>
-  <si>
-    <t>29-07-2026</t>
-  </si>
-  <si>
-    <t>21-07-2026</t>
-  </si>
-  <si>
-    <t>07-07-2026</t>
-  </si>
-  <si>
-    <t>30-06-2026</t>
-  </si>
-  <si>
-    <t>20-07-2026</t>
-  </si>
-  <si>
-    <t>10-07-2026</t>
-  </si>
-  <si>
-    <t>23-07-2026</t>
-  </si>
-  <si>
-    <t>27-07-2026</t>
-  </si>
-  <si>
-    <t>08-07-2026</t>
-  </si>
-  <si>
-    <t>22-07-2026</t>
-  </si>
-  <si>
-    <t>06-07-2026</t>
-  </si>
-  <si>
-    <t>24-07-2026</t>
-  </si>
-  <si>
-    <t>25-07-2026</t>
-  </si>
-  <si>
-    <t>26-07-2026</t>
-  </si>
-  <si>
-    <t>03-07-2026</t>
   </si>
 </sst>
 </file>
@@ -2736,7 +2739,7 @@
         <v>689</v>
       </c>
       <c r="O2">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -2801,7 +2804,7 @@
         <v>690</v>
       </c>
       <c r="O3">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="P3">
         <v>0</v>
@@ -2866,7 +2869,7 @@
         <v>691</v>
       </c>
       <c r="O4">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="P4">
         <v>1</v>
@@ -2931,7 +2934,7 @@
         <v>691</v>
       </c>
       <c r="O5">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="P5">
         <v>1</v>
@@ -2996,7 +2999,7 @@
         <v>692</v>
       </c>
       <c r="O6">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -3061,7 +3064,7 @@
         <v>693</v>
       </c>
       <c r="O7">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -3126,7 +3129,7 @@
         <v>694</v>
       </c>
       <c r="O8">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -3191,7 +3194,7 @@
         <v>695</v>
       </c>
       <c r="O9">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -3256,7 +3259,7 @@
         <v>696</v>
       </c>
       <c r="O10">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="P10">
         <v>1</v>
@@ -3321,7 +3324,7 @@
         <v>689</v>
       </c>
       <c r="O11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="P11">
         <v>0</v>
@@ -3386,7 +3389,7 @@
         <v>697</v>
       </c>
       <c r="O12">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -3451,7 +3454,7 @@
         <v>698</v>
       </c>
       <c r="O13">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="P13">
         <v>1</v>
@@ -3516,7 +3519,7 @@
         <v>699</v>
       </c>
       <c r="O14">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="P14">
         <v>1</v>
@@ -3581,7 +3584,7 @@
         <v>699</v>
       </c>
       <c r="O15">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -3646,7 +3649,7 @@
         <v>700</v>
       </c>
       <c r="O16">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="P16">
         <v>3</v>
@@ -3711,7 +3714,7 @@
         <v>692</v>
       </c>
       <c r="O17">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="P17">
         <v>0</v>
@@ -3776,7 +3779,7 @@
         <v>692</v>
       </c>
       <c r="O18">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="P18">
         <v>0</v>
@@ -3841,7 +3844,7 @@
         <v>691</v>
       </c>
       <c r="O19">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="P19">
         <v>1</v>
@@ -3906,7 +3909,7 @@
         <v>695</v>
       </c>
       <c r="O20">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="P20">
         <v>1</v>
@@ -3971,7 +3974,7 @@
         <v>701</v>
       </c>
       <c r="O21">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="P21">
         <v>0</v>
@@ -4036,7 +4039,7 @@
         <v>702</v>
       </c>
       <c r="O22">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="P22">
         <v>0</v>
@@ -4101,7 +4104,7 @@
         <v>702</v>
       </c>
       <c r="O23">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="P23">
         <v>2</v>
@@ -4166,7 +4169,7 @@
         <v>691</v>
       </c>
       <c r="O24">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="P24">
         <v>0</v>
@@ -4231,7 +4234,7 @@
         <v>691</v>
       </c>
       <c r="O25">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="P25">
         <v>0</v>
@@ -4296,7 +4299,7 @@
         <v>692</v>
       </c>
       <c r="O26">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="P26">
         <v>1</v>
@@ -4361,7 +4364,7 @@
         <v>703</v>
       </c>
       <c r="O27">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="P27">
         <v>2</v>
@@ -4426,7 +4429,7 @@
         <v>698</v>
       </c>
       <c r="O28">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -4491,7 +4494,7 @@
         <v>700</v>
       </c>
       <c r="O29">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="P29">
         <v>1</v>
@@ -4556,7 +4559,7 @@
         <v>704</v>
       </c>
       <c r="O30">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="P30">
         <v>0</v>
@@ -4574,7 +4577,7 @@
         <v>738</v>
       </c>
       <c r="U30">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:21">
@@ -4621,7 +4624,7 @@
         <v>695</v>
       </c>
       <c r="O31">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="P31">
         <v>0</v>
@@ -4686,7 +4689,7 @@
         <v>689</v>
       </c>
       <c r="O32">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="P32">
         <v>1</v>
@@ -4751,7 +4754,7 @@
         <v>689</v>
       </c>
       <c r="O33">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="P33">
         <v>1</v>
@@ -4816,7 +4819,7 @@
         <v>702</v>
       </c>
       <c r="O34">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="P34">
         <v>0</v>
@@ -4881,7 +4884,7 @@
         <v>697</v>
       </c>
       <c r="O35">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="P35">
         <v>0</v>
@@ -4946,7 +4949,7 @@
         <v>705</v>
       </c>
       <c r="O36">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="P36">
         <v>0</v>
@@ -4964,7 +4967,7 @@
         <v>739</v>
       </c>
       <c r="U36">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:21">
@@ -5011,7 +5014,7 @@
         <v>706</v>
       </c>
       <c r="O37">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="P37">
         <v>0</v>
@@ -5076,7 +5079,7 @@
         <v>707</v>
       </c>
       <c r="O38">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="P38">
         <v>2</v>
@@ -5141,7 +5144,7 @@
         <v>693</v>
       </c>
       <c r="O39">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="P39">
         <v>0</v>
@@ -5206,7 +5209,7 @@
         <v>698</v>
       </c>
       <c r="O40">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="P40">
         <v>2</v>
@@ -5271,7 +5274,7 @@
         <v>708</v>
       </c>
       <c r="O41">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="P41">
         <v>0</v>
@@ -5336,7 +5339,7 @@
         <v>709</v>
       </c>
       <c r="O42">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="P42">
         <v>3</v>
@@ -5401,7 +5404,7 @@
         <v>692</v>
       </c>
       <c r="O43">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="P43">
         <v>2</v>
@@ -5466,7 +5469,7 @@
         <v>694</v>
       </c>
       <c r="O44">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="P44">
         <v>0</v>
@@ -5531,7 +5534,7 @@
         <v>707</v>
       </c>
       <c r="O45">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="P45">
         <v>0</v>
@@ -5596,7 +5599,7 @@
         <v>709</v>
       </c>
       <c r="O46">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="P46">
         <v>0</v>
@@ -5661,7 +5664,7 @@
         <v>698</v>
       </c>
       <c r="O47">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="P47">
         <v>0</v>
@@ -5726,7 +5729,7 @@
         <v>705</v>
       </c>
       <c r="O48">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="P48">
         <v>0</v>
@@ -5744,7 +5747,7 @@
         <v>739</v>
       </c>
       <c r="U48">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:21">
@@ -5791,7 +5794,7 @@
         <v>710</v>
       </c>
       <c r="O49">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="P49">
         <v>1</v>
@@ -5856,7 +5859,7 @@
         <v>689</v>
       </c>
       <c r="O50">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="P50">
         <v>2</v>
@@ -5921,7 +5924,7 @@
         <v>698</v>
       </c>
       <c r="O51">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="P51">
         <v>0</v>
@@ -5986,7 +5989,7 @@
         <v>702</v>
       </c>
       <c r="O52">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="P52">
         <v>0</v>
@@ -6051,7 +6054,7 @@
         <v>702</v>
       </c>
       <c r="O53">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="P53">
         <v>1</v>
@@ -6116,7 +6119,7 @@
         <v>693</v>
       </c>
       <c r="O54">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="P54">
         <v>0</v>
@@ -6181,7 +6184,7 @@
         <v>706</v>
       </c>
       <c r="O55">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="P55">
         <v>1</v>
@@ -6246,7 +6249,7 @@
         <v>700</v>
       </c>
       <c r="O56">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="P56">
         <v>0</v>
@@ -6311,7 +6314,7 @@
         <v>701</v>
       </c>
       <c r="O57">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="P57">
         <v>0</v>
@@ -6376,7 +6379,7 @@
         <v>707</v>
       </c>
       <c r="O58">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="P58">
         <v>0</v>
@@ -6441,7 +6444,7 @@
         <v>711</v>
       </c>
       <c r="O59">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="P59">
         <v>2</v>
@@ -6506,7 +6509,7 @@
         <v>712</v>
       </c>
       <c r="O60">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="P60">
         <v>1</v>
@@ -6524,7 +6527,7 @@
         <v>746</v>
       </c>
       <c r="U60">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:21">
@@ -6571,7 +6574,7 @@
         <v>689</v>
       </c>
       <c r="O61">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="P61">
         <v>1</v>
@@ -6636,7 +6639,7 @@
         <v>713</v>
       </c>
       <c r="O62">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="P62">
         <v>1</v>
@@ -6701,7 +6704,7 @@
         <v>710</v>
       </c>
       <c r="O63">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="P63">
         <v>1</v>
@@ -6766,7 +6769,7 @@
         <v>697</v>
       </c>
       <c r="O64">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="P64">
         <v>0</v>
@@ -6831,7 +6834,7 @@
         <v>707</v>
       </c>
       <c r="O65">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="P65">
         <v>0</v>
@@ -6896,7 +6899,7 @@
         <v>708</v>
       </c>
       <c r="O66">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="P66">
         <v>2</v>
@@ -6961,7 +6964,7 @@
         <v>693</v>
       </c>
       <c r="O67">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="P67">
         <v>4</v>
@@ -7026,7 +7029,7 @@
         <v>695</v>
       </c>
       <c r="O68">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="P68">
         <v>0</v>
@@ -7091,7 +7094,7 @@
         <v>695</v>
       </c>
       <c r="O69">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="P69">
         <v>0</v>
@@ -7156,7 +7159,7 @@
         <v>710</v>
       </c>
       <c r="O70">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="P70">
         <v>2</v>
@@ -7221,7 +7224,7 @@
         <v>702</v>
       </c>
       <c r="O71">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="P71">
         <v>1</v>
@@ -7286,7 +7289,7 @@
         <v>695</v>
       </c>
       <c r="O72">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="P72">
         <v>0</v>
@@ -7351,7 +7354,7 @@
         <v>705</v>
       </c>
       <c r="O73">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="P73">
         <v>0</v>
@@ -7369,7 +7372,7 @@
         <v>739</v>
       </c>
       <c r="U73">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:21">
@@ -7416,7 +7419,7 @@
         <v>694</v>
       </c>
       <c r="O74">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="P74">
         <v>3</v>
@@ -7481,7 +7484,7 @@
         <v>714</v>
       </c>
       <c r="O75">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P75">
         <v>0</v>
@@ -7546,7 +7549,7 @@
         <v>708</v>
       </c>
       <c r="O76">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="P76">
         <v>3</v>
@@ -7611,7 +7614,7 @@
         <v>711</v>
       </c>
       <c r="O77">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="P77">
         <v>0</v>
@@ -7676,7 +7679,7 @@
         <v>710</v>
       </c>
       <c r="O78">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="P78">
         <v>2</v>
@@ -7741,7 +7744,7 @@
         <v>707</v>
       </c>
       <c r="O79">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="P79">
         <v>0</v>
@@ -7806,7 +7809,7 @@
         <v>715</v>
       </c>
       <c r="O80">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="P80">
         <v>2</v>
@@ -7871,7 +7874,7 @@
         <v>714</v>
       </c>
       <c r="O81">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P81">
         <v>1</v>
@@ -7936,7 +7939,7 @@
         <v>716</v>
       </c>
       <c r="O82">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="P82">
         <v>1</v>
@@ -7951,10 +7954,10 @@
         <v>0</v>
       </c>
       <c r="T82" t="s">
-        <v>739</v>
+        <v>750</v>
       </c>
       <c r="U82">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:21">
@@ -8001,7 +8004,7 @@
         <v>717</v>
       </c>
       <c r="O83">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="P83">
         <v>0</v>
@@ -8016,7 +8019,7 @@
         <v>1</v>
       </c>
       <c r="T83" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="U83">
         <v>0</v>
@@ -8066,7 +8069,7 @@
         <v>716</v>
       </c>
       <c r="O84">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="P84">
         <v>2</v>
@@ -8081,10 +8084,10 @@
         <v>1</v>
       </c>
       <c r="T84" t="s">
-        <v>739</v>
+        <v>750</v>
       </c>
       <c r="U84">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:21">
@@ -8131,7 +8134,7 @@
         <v>698</v>
       </c>
       <c r="O85">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="P85">
         <v>4</v>
@@ -8196,7 +8199,7 @@
         <v>698</v>
       </c>
       <c r="O86">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="P86">
         <v>1</v>
@@ -8261,7 +8264,7 @@
         <v>694</v>
       </c>
       <c r="O87">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="P87">
         <v>4</v>
@@ -8326,7 +8329,7 @@
         <v>691</v>
       </c>
       <c r="O88">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="P88">
         <v>0</v>
@@ -8391,7 +8394,7 @@
         <v>707</v>
       </c>
       <c r="O89">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="P89">
         <v>0</v>
@@ -8456,7 +8459,7 @@
         <v>692</v>
       </c>
       <c r="O90">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="P90">
         <v>0</v>
@@ -8521,7 +8524,7 @@
         <v>702</v>
       </c>
       <c r="O91">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="P91">
         <v>0</v>
@@ -8586,7 +8589,7 @@
         <v>710</v>
       </c>
       <c r="O92">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="P92">
         <v>0</v>
@@ -8651,7 +8654,7 @@
         <v>697</v>
       </c>
       <c r="O93">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="P93">
         <v>0</v>
@@ -8716,7 +8719,7 @@
         <v>703</v>
       </c>
       <c r="O94">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="P94">
         <v>1</v>
@@ -8781,7 +8784,7 @@
         <v>691</v>
       </c>
       <c r="O95">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="P95">
         <v>0</v>
@@ -8846,7 +8849,7 @@
         <v>710</v>
       </c>
       <c r="O96">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="P96">
         <v>2</v>
@@ -8911,7 +8914,7 @@
         <v>711</v>
       </c>
       <c r="O97">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="P97">
         <v>0</v>
@@ -8976,7 +8979,7 @@
         <v>696</v>
       </c>
       <c r="O98">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="P98">
         <v>1</v>
@@ -9041,7 +9044,7 @@
         <v>713</v>
       </c>
       <c r="O99">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="P99">
         <v>0</v>
@@ -9106,7 +9109,7 @@
         <v>706</v>
       </c>
       <c r="O100">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="P100">
         <v>0</v>
@@ -9171,7 +9174,7 @@
         <v>708</v>
       </c>
       <c r="O101">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="P101">
         <v>1</v>

</xml_diff>

<commit_message>
Update client attention, missed SIP status, proposals and lead management
</commit_message>
<xml_diff>
--- a/backend/data/sip_advisor_enriched_preview.xlsx
+++ b/backend/data/sip_advisor_enriched_preview.xlsx
@@ -2875,7 +2875,7 @@
         <v>1</v>
       </c>
       <c r="Q4" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R4" t="s">
         <v>721</v>
@@ -2940,7 +2940,7 @@
         <v>1</v>
       </c>
       <c r="Q5" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R5" t="s">
         <v>721</v>
@@ -3265,7 +3265,7 @@
         <v>1</v>
       </c>
       <c r="Q10" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R10" t="s">
         <v>721</v>
@@ -3460,7 +3460,7 @@
         <v>1</v>
       </c>
       <c r="Q13" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R13" t="s">
         <v>721</v>
@@ -3525,7 +3525,7 @@
         <v>1</v>
       </c>
       <c r="Q14" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R14" t="s">
         <v>721</v>
@@ -3850,7 +3850,7 @@
         <v>1</v>
       </c>
       <c r="Q19" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R19" t="s">
         <v>721</v>
@@ -3915,7 +3915,7 @@
         <v>1</v>
       </c>
       <c r="Q20" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R20" t="s">
         <v>721</v>
@@ -4110,7 +4110,7 @@
         <v>2</v>
       </c>
       <c r="Q23" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R23" t="s">
         <v>721</v>
@@ -4305,7 +4305,7 @@
         <v>1</v>
       </c>
       <c r="Q26" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R26" t="s">
         <v>721</v>
@@ -4370,7 +4370,7 @@
         <v>2</v>
       </c>
       <c r="Q27" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R27" t="s">
         <v>721</v>
@@ -4500,7 +4500,7 @@
         <v>1</v>
       </c>
       <c r="Q29" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R29" t="s">
         <v>721</v>
@@ -4695,7 +4695,7 @@
         <v>1</v>
       </c>
       <c r="Q32" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R32" t="s">
         <v>721</v>
@@ -4760,7 +4760,7 @@
         <v>1</v>
       </c>
       <c r="Q33" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R33" t="s">
         <v>721</v>
@@ -5085,7 +5085,7 @@
         <v>2</v>
       </c>
       <c r="Q38" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R38" t="s">
         <v>721</v>
@@ -5215,7 +5215,7 @@
         <v>2</v>
       </c>
       <c r="Q40" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R40" t="s">
         <v>721</v>
@@ -5410,7 +5410,7 @@
         <v>2</v>
       </c>
       <c r="Q43" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R43" t="s">
         <v>721</v>
@@ -5800,7 +5800,7 @@
         <v>1</v>
       </c>
       <c r="Q49" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R49" t="s">
         <v>721</v>
@@ -5865,7 +5865,7 @@
         <v>2</v>
       </c>
       <c r="Q50" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R50" t="s">
         <v>721</v>
@@ -6060,7 +6060,7 @@
         <v>1</v>
       </c>
       <c r="Q53" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R53" t="s">
         <v>721</v>
@@ -6190,7 +6190,7 @@
         <v>1</v>
       </c>
       <c r="Q55" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R55" t="s">
         <v>721</v>
@@ -6450,7 +6450,7 @@
         <v>2</v>
       </c>
       <c r="Q59" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R59" t="s">
         <v>721</v>
@@ -6515,7 +6515,7 @@
         <v>1</v>
       </c>
       <c r="Q60" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R60" t="s">
         <v>721</v>
@@ -6580,7 +6580,7 @@
         <v>1</v>
       </c>
       <c r="Q61" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R61" t="s">
         <v>721</v>
@@ -6645,7 +6645,7 @@
         <v>1</v>
       </c>
       <c r="Q62" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R62" t="s">
         <v>721</v>
@@ -6710,7 +6710,7 @@
         <v>1</v>
       </c>
       <c r="Q63" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R63" t="s">
         <v>721</v>
@@ -6905,7 +6905,7 @@
         <v>2</v>
       </c>
       <c r="Q66" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R66" t="s">
         <v>721</v>
@@ -7165,7 +7165,7 @@
         <v>2</v>
       </c>
       <c r="Q70" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R70" t="s">
         <v>721</v>
@@ -7230,7 +7230,7 @@
         <v>1</v>
       </c>
       <c r="Q71" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R71" t="s">
         <v>721</v>
@@ -7685,7 +7685,7 @@
         <v>2</v>
       </c>
       <c r="Q78" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R78" t="s">
         <v>721</v>
@@ -7815,7 +7815,7 @@
         <v>2</v>
       </c>
       <c r="Q80" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R80" t="s">
         <v>721</v>
@@ -7880,7 +7880,7 @@
         <v>1</v>
       </c>
       <c r="Q81" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R81" t="s">
         <v>721</v>
@@ -7945,7 +7945,7 @@
         <v>1</v>
       </c>
       <c r="Q82" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R82" t="s">
         <v>721</v>
@@ -8075,7 +8075,7 @@
         <v>2</v>
       </c>
       <c r="Q84" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R84" t="s">
         <v>721</v>
@@ -8205,7 +8205,7 @@
         <v>1</v>
       </c>
       <c r="Q86" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R86" t="s">
         <v>721</v>
@@ -8725,7 +8725,7 @@
         <v>1</v>
       </c>
       <c r="Q94" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R94" t="s">
         <v>721</v>
@@ -8855,7 +8855,7 @@
         <v>2</v>
       </c>
       <c r="Q96" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R96" t="s">
         <v>721</v>
@@ -8985,7 +8985,7 @@
         <v>1</v>
       </c>
       <c r="Q98" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R98" t="s">
         <v>721</v>
@@ -9180,7 +9180,7 @@
         <v>1</v>
       </c>
       <c r="Q101" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="R101" t="s">
         <v>721</v>

</xml_diff>

<commit_message>
Fix missing SIP fields in raw/manual-add path, fix status logic, aggregate attention widget
</commit_message>
<xml_diff>
--- a/backend/data/sip_advisor_enriched_preview.xlsx
+++ b/backend/data/sip_advisor_enriched_preview.xlsx
@@ -2092,19 +2092,121 @@
     <t>28-08-2026</t>
   </si>
   <si>
+    <t>12-09-2026</t>
+  </si>
+  <si>
+    <t>17-08-2026</t>
+  </si>
+  <si>
+    <t>14-09-2026</t>
+  </si>
+  <si>
+    <t>02-09-2026</t>
+  </si>
+  <si>
+    <t>18-08-2026</t>
+  </si>
+  <si>
+    <t>13-09-2026</t>
+  </si>
+  <si>
+    <t>11-09-2026</t>
+  </si>
+  <si>
+    <t>15-09-2026</t>
+  </si>
+  <si>
+    <t>05-09-2026</t>
+  </si>
+  <si>
+    <t>04-09-2026</t>
+  </si>
+  <si>
+    <t>29-08-2026</t>
+  </si>
+  <si>
+    <t>21-08-2026</t>
+  </si>
+  <si>
+    <t>07-09-2026</t>
+  </si>
+  <si>
+    <t>30-08-2026</t>
+  </si>
+  <si>
+    <t>20-08-2026</t>
+  </si>
+  <si>
+    <t>10-09-2026</t>
+  </si>
+  <si>
+    <t>23-08-2026</t>
+  </si>
+  <si>
+    <t>27-08-2026</t>
+  </si>
+  <si>
+    <t>08-09-2026</t>
+  </si>
+  <si>
+    <t>22-08-2026</t>
+  </si>
+  <si>
+    <t>06-09-2026</t>
+  </si>
+  <si>
+    <t>24-08-2026</t>
+  </si>
+  <si>
+    <t>25-08-2026</t>
+  </si>
+  <si>
+    <t>26-08-2026</t>
+  </si>
+  <si>
+    <t>31-08-2026</t>
+  </si>
+  <si>
+    <t>03-09-2026</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Missed</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>19-07-2026</t>
+  </si>
+  <si>
+    <t>16-07-2026</t>
+  </si>
+  <si>
+    <t>28-07-2026</t>
+  </si>
+  <si>
     <t>12-08-2026</t>
   </si>
   <si>
-    <t>17-08-2026</t>
+    <t>17-07-2026</t>
   </si>
   <si>
     <t>14-08-2026</t>
   </si>
   <si>
-    <t>02-09-2026</t>
-  </si>
-  <si>
-    <t>18-08-2026</t>
+    <t>02-08-2026</t>
+  </si>
+  <si>
+    <t>18-07-2026</t>
   </si>
   <si>
     <t>13-08-2026</t>
@@ -2116,145 +2218,43 @@
     <t>15-08-2026</t>
   </si>
   <si>
-    <t>05-09-2026</t>
-  </si>
-  <si>
-    <t>04-09-2026</t>
-  </si>
-  <si>
-    <t>29-08-2026</t>
-  </si>
-  <si>
-    <t>21-08-2026</t>
+    <t>05-08-2026</t>
+  </si>
+  <si>
+    <t>04-08-2026</t>
+  </si>
+  <si>
+    <t>29-07-2026</t>
+  </si>
+  <si>
+    <t>21-07-2026</t>
   </si>
   <si>
     <t>07-08-2026</t>
   </si>
   <si>
-    <t>30-08-2026</t>
-  </si>
-  <si>
-    <t>20-08-2026</t>
+    <t>30-07-2026</t>
+  </si>
+  <si>
+    <t>20-07-2026</t>
   </si>
   <si>
     <t>10-08-2026</t>
   </si>
   <si>
-    <t>23-08-2026</t>
-  </si>
-  <si>
-    <t>27-08-2026</t>
+    <t>23-07-2026</t>
+  </si>
+  <si>
+    <t>27-07-2026</t>
   </si>
   <si>
     <t>08-08-2026</t>
   </si>
   <si>
-    <t>22-08-2026</t>
+    <t>22-07-2026</t>
   </si>
   <si>
     <t>06-08-2026</t>
-  </si>
-  <si>
-    <t>24-08-2026</t>
-  </si>
-  <si>
-    <t>25-08-2026</t>
-  </si>
-  <si>
-    <t>26-08-2026</t>
-  </si>
-  <si>
-    <t>31-08-2026</t>
-  </si>
-  <si>
-    <t>03-09-2026</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Missed</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>19-07-2026</t>
-  </si>
-  <si>
-    <t>16-07-2026</t>
-  </si>
-  <si>
-    <t>28-07-2026</t>
-  </si>
-  <si>
-    <t>12-07-2026</t>
-  </si>
-  <si>
-    <t>17-07-2026</t>
-  </si>
-  <si>
-    <t>14-07-2026</t>
-  </si>
-  <si>
-    <t>02-08-2026</t>
-  </si>
-  <si>
-    <t>18-07-2026</t>
-  </si>
-  <si>
-    <t>13-07-2026</t>
-  </si>
-  <si>
-    <t>11-07-2026</t>
-  </si>
-  <si>
-    <t>15-07-2026</t>
-  </si>
-  <si>
-    <t>05-08-2026</t>
-  </si>
-  <si>
-    <t>04-08-2026</t>
-  </si>
-  <si>
-    <t>29-07-2026</t>
-  </si>
-  <si>
-    <t>21-07-2026</t>
-  </si>
-  <si>
-    <t>07-07-2026</t>
-  </si>
-  <si>
-    <t>30-07-2026</t>
-  </si>
-  <si>
-    <t>20-07-2026</t>
-  </si>
-  <si>
-    <t>10-07-2026</t>
-  </si>
-  <si>
-    <t>23-07-2026</t>
-  </si>
-  <si>
-    <t>27-07-2026</t>
-  </si>
-  <si>
-    <t>08-07-2026</t>
-  </si>
-  <si>
-    <t>22-07-2026</t>
-  </si>
-  <si>
-    <t>06-07-2026</t>
   </si>
   <si>
     <t>24-07-2026</t>
@@ -2739,7 +2739,7 @@
         <v>689</v>
       </c>
       <c r="O2">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>690</v>
       </c>
       <c r="O3">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="P3">
         <v>0</v>
@@ -2822,7 +2822,7 @@
         <v>724</v>
       </c>
       <c r="U3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -2869,13 +2869,13 @@
         <v>691</v>
       </c>
       <c r="O4">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="P4">
         <v>1</v>
       </c>
       <c r="Q4" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R4" t="s">
         <v>721</v>
@@ -2934,13 +2934,13 @@
         <v>691</v>
       </c>
       <c r="O5">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="P5">
         <v>1</v>
       </c>
       <c r="Q5" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R5" t="s">
         <v>721</v>
@@ -2999,7 +2999,7 @@
         <v>692</v>
       </c>
       <c r="O6">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -3064,7 +3064,7 @@
         <v>693</v>
       </c>
       <c r="O7">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -3082,7 +3082,7 @@
         <v>727</v>
       </c>
       <c r="U7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:21">
@@ -3129,7 +3129,7 @@
         <v>694</v>
       </c>
       <c r="O8">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -3194,7 +3194,7 @@
         <v>695</v>
       </c>
       <c r="O9">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -3259,13 +3259,13 @@
         <v>696</v>
       </c>
       <c r="O10">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="P10">
         <v>1</v>
       </c>
       <c r="Q10" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R10" t="s">
         <v>721</v>
@@ -3324,7 +3324,7 @@
         <v>689</v>
       </c>
       <c r="O11">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="P11">
         <v>0</v>
@@ -3389,7 +3389,7 @@
         <v>697</v>
       </c>
       <c r="O12">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -3454,13 +3454,13 @@
         <v>698</v>
       </c>
       <c r="O13">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="P13">
         <v>1</v>
       </c>
       <c r="Q13" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R13" t="s">
         <v>721</v>
@@ -3519,13 +3519,13 @@
         <v>699</v>
       </c>
       <c r="O14">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="P14">
         <v>1</v>
       </c>
       <c r="Q14" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R14" t="s">
         <v>721</v>
@@ -3584,7 +3584,7 @@
         <v>699</v>
       </c>
       <c r="O15">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -3649,7 +3649,7 @@
         <v>700</v>
       </c>
       <c r="O16">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="P16">
         <v>3</v>
@@ -3714,7 +3714,7 @@
         <v>692</v>
       </c>
       <c r="O17">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="P17">
         <v>0</v>
@@ -3779,7 +3779,7 @@
         <v>692</v>
       </c>
       <c r="O18">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="P18">
         <v>0</v>
@@ -3844,13 +3844,13 @@
         <v>691</v>
       </c>
       <c r="O19">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="P19">
         <v>1</v>
       </c>
       <c r="Q19" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R19" t="s">
         <v>721</v>
@@ -3909,13 +3909,13 @@
         <v>695</v>
       </c>
       <c r="O20">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="P20">
         <v>1</v>
       </c>
       <c r="Q20" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R20" t="s">
         <v>721</v>
@@ -3974,7 +3974,7 @@
         <v>701</v>
       </c>
       <c r="O21">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="P21">
         <v>0</v>
@@ -4039,7 +4039,7 @@
         <v>702</v>
       </c>
       <c r="O22">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="P22">
         <v>0</v>
@@ -4104,13 +4104,13 @@
         <v>702</v>
       </c>
       <c r="O23">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="P23">
         <v>2</v>
       </c>
       <c r="Q23" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R23" t="s">
         <v>721</v>
@@ -4169,7 +4169,7 @@
         <v>691</v>
       </c>
       <c r="O24">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="P24">
         <v>0</v>
@@ -4234,7 +4234,7 @@
         <v>691</v>
       </c>
       <c r="O25">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="P25">
         <v>0</v>
@@ -4299,13 +4299,13 @@
         <v>692</v>
       </c>
       <c r="O26">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="P26">
         <v>1</v>
       </c>
       <c r="Q26" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R26" t="s">
         <v>721</v>
@@ -4364,13 +4364,13 @@
         <v>703</v>
       </c>
       <c r="O27">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="P27">
         <v>2</v>
       </c>
       <c r="Q27" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R27" t="s">
         <v>721</v>
@@ -4429,7 +4429,7 @@
         <v>698</v>
       </c>
       <c r="O28">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -4494,13 +4494,13 @@
         <v>700</v>
       </c>
       <c r="O29">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="P29">
         <v>1</v>
       </c>
       <c r="Q29" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R29" t="s">
         <v>721</v>
@@ -4559,7 +4559,7 @@
         <v>704</v>
       </c>
       <c r="O30">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="P30">
         <v>0</v>
@@ -4577,7 +4577,7 @@
         <v>738</v>
       </c>
       <c r="U30">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:21">
@@ -4624,7 +4624,7 @@
         <v>695</v>
       </c>
       <c r="O31">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="P31">
         <v>0</v>
@@ -4689,13 +4689,13 @@
         <v>689</v>
       </c>
       <c r="O32">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="P32">
         <v>1</v>
       </c>
       <c r="Q32" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R32" t="s">
         <v>721</v>
@@ -4754,13 +4754,13 @@
         <v>689</v>
       </c>
       <c r="O33">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="P33">
         <v>1</v>
       </c>
       <c r="Q33" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R33" t="s">
         <v>721</v>
@@ -4819,7 +4819,7 @@
         <v>702</v>
       </c>
       <c r="O34">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="P34">
         <v>0</v>
@@ -4884,7 +4884,7 @@
         <v>697</v>
       </c>
       <c r="O35">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="P35">
         <v>0</v>
@@ -4949,7 +4949,7 @@
         <v>705</v>
       </c>
       <c r="O36">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="P36">
         <v>0</v>
@@ -5014,7 +5014,7 @@
         <v>706</v>
       </c>
       <c r="O37">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="P37">
         <v>0</v>
@@ -5079,13 +5079,13 @@
         <v>707</v>
       </c>
       <c r="O38">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="P38">
         <v>2</v>
       </c>
       <c r="Q38" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R38" t="s">
         <v>721</v>
@@ -5144,7 +5144,7 @@
         <v>693</v>
       </c>
       <c r="O39">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="P39">
         <v>0</v>
@@ -5162,7 +5162,7 @@
         <v>727</v>
       </c>
       <c r="U39">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:21">
@@ -5209,13 +5209,13 @@
         <v>698</v>
       </c>
       <c r="O40">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="P40">
         <v>2</v>
       </c>
       <c r="Q40" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R40" t="s">
         <v>721</v>
@@ -5274,7 +5274,7 @@
         <v>708</v>
       </c>
       <c r="O41">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="P41">
         <v>0</v>
@@ -5339,7 +5339,7 @@
         <v>709</v>
       </c>
       <c r="O42">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="P42">
         <v>3</v>
@@ -5404,13 +5404,13 @@
         <v>692</v>
       </c>
       <c r="O43">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="P43">
         <v>2</v>
       </c>
       <c r="Q43" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R43" t="s">
         <v>721</v>
@@ -5469,7 +5469,7 @@
         <v>694</v>
       </c>
       <c r="O44">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="P44">
         <v>0</v>
@@ -5534,7 +5534,7 @@
         <v>707</v>
       </c>
       <c r="O45">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="P45">
         <v>0</v>
@@ -5599,7 +5599,7 @@
         <v>709</v>
       </c>
       <c r="O46">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="P46">
         <v>0</v>
@@ -5664,7 +5664,7 @@
         <v>698</v>
       </c>
       <c r="O47">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="P47">
         <v>0</v>
@@ -5729,7 +5729,7 @@
         <v>705</v>
       </c>
       <c r="O48">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="P48">
         <v>0</v>
@@ -5794,13 +5794,13 @@
         <v>710</v>
       </c>
       <c r="O49">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="P49">
         <v>1</v>
       </c>
       <c r="Q49" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R49" t="s">
         <v>721</v>
@@ -5859,13 +5859,13 @@
         <v>689</v>
       </c>
       <c r="O50">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="P50">
         <v>2</v>
       </c>
       <c r="Q50" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R50" t="s">
         <v>721</v>
@@ -5924,7 +5924,7 @@
         <v>698</v>
       </c>
       <c r="O51">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="P51">
         <v>0</v>
@@ -5989,7 +5989,7 @@
         <v>702</v>
       </c>
       <c r="O52">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="P52">
         <v>0</v>
@@ -6054,13 +6054,13 @@
         <v>702</v>
       </c>
       <c r="O53">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="P53">
         <v>1</v>
       </c>
       <c r="Q53" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R53" t="s">
         <v>721</v>
@@ -6119,7 +6119,7 @@
         <v>693</v>
       </c>
       <c r="O54">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="P54">
         <v>0</v>
@@ -6137,7 +6137,7 @@
         <v>727</v>
       </c>
       <c r="U54">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:21">
@@ -6184,13 +6184,13 @@
         <v>706</v>
       </c>
       <c r="O55">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="P55">
         <v>1</v>
       </c>
       <c r="Q55" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R55" t="s">
         <v>721</v>
@@ -6249,7 +6249,7 @@
         <v>700</v>
       </c>
       <c r="O56">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="P56">
         <v>0</v>
@@ -6314,7 +6314,7 @@
         <v>701</v>
       </c>
       <c r="O57">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="P57">
         <v>0</v>
@@ -6379,7 +6379,7 @@
         <v>707</v>
       </c>
       <c r="O58">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="P58">
         <v>0</v>
@@ -6444,13 +6444,13 @@
         <v>711</v>
       </c>
       <c r="O59">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="P59">
         <v>2</v>
       </c>
       <c r="Q59" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R59" t="s">
         <v>721</v>
@@ -6509,13 +6509,13 @@
         <v>712</v>
       </c>
       <c r="O60">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="P60">
         <v>1</v>
       </c>
       <c r="Q60" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R60" t="s">
         <v>721</v>
@@ -6527,7 +6527,7 @@
         <v>746</v>
       </c>
       <c r="U60">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:21">
@@ -6574,13 +6574,13 @@
         <v>689</v>
       </c>
       <c r="O61">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="P61">
         <v>1</v>
       </c>
       <c r="Q61" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R61" t="s">
         <v>721</v>
@@ -6639,13 +6639,13 @@
         <v>713</v>
       </c>
       <c r="O62">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="P62">
         <v>1</v>
       </c>
       <c r="Q62" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R62" t="s">
         <v>721</v>
@@ -6704,13 +6704,13 @@
         <v>710</v>
       </c>
       <c r="O63">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="P63">
         <v>1</v>
       </c>
       <c r="Q63" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R63" t="s">
         <v>721</v>
@@ -6769,7 +6769,7 @@
         <v>697</v>
       </c>
       <c r="O64">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="P64">
         <v>0</v>
@@ -6834,7 +6834,7 @@
         <v>707</v>
       </c>
       <c r="O65">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="P65">
         <v>0</v>
@@ -6899,13 +6899,13 @@
         <v>708</v>
       </c>
       <c r="O66">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="P66">
         <v>2</v>
       </c>
       <c r="Q66" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R66" t="s">
         <v>721</v>
@@ -6964,7 +6964,7 @@
         <v>693</v>
       </c>
       <c r="O67">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="P67">
         <v>4</v>
@@ -6982,7 +6982,7 @@
         <v>727</v>
       </c>
       <c r="U67">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:21">
@@ -7029,7 +7029,7 @@
         <v>695</v>
       </c>
       <c r="O68">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="P68">
         <v>0</v>
@@ -7094,7 +7094,7 @@
         <v>695</v>
       </c>
       <c r="O69">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="P69">
         <v>0</v>
@@ -7159,13 +7159,13 @@
         <v>710</v>
       </c>
       <c r="O70">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="P70">
         <v>2</v>
       </c>
       <c r="Q70" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R70" t="s">
         <v>721</v>
@@ -7224,13 +7224,13 @@
         <v>702</v>
       </c>
       <c r="O71">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="P71">
         <v>1</v>
       </c>
       <c r="Q71" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R71" t="s">
         <v>721</v>
@@ -7289,7 +7289,7 @@
         <v>695</v>
       </c>
       <c r="O72">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="P72">
         <v>0</v>
@@ -7354,7 +7354,7 @@
         <v>705</v>
       </c>
       <c r="O73">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="P73">
         <v>0</v>
@@ -7419,7 +7419,7 @@
         <v>694</v>
       </c>
       <c r="O74">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="P74">
         <v>3</v>
@@ -7484,7 +7484,7 @@
         <v>714</v>
       </c>
       <c r="O75">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="P75">
         <v>0</v>
@@ -7549,7 +7549,7 @@
         <v>708</v>
       </c>
       <c r="O76">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="P76">
         <v>3</v>
@@ -7614,7 +7614,7 @@
         <v>711</v>
       </c>
       <c r="O77">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="P77">
         <v>0</v>
@@ -7679,13 +7679,13 @@
         <v>710</v>
       </c>
       <c r="O78">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="P78">
         <v>2</v>
       </c>
       <c r="Q78" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R78" t="s">
         <v>721</v>
@@ -7744,7 +7744,7 @@
         <v>707</v>
       </c>
       <c r="O79">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="P79">
         <v>0</v>
@@ -7809,13 +7809,13 @@
         <v>715</v>
       </c>
       <c r="O80">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="P80">
         <v>2</v>
       </c>
       <c r="Q80" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R80" t="s">
         <v>721</v>
@@ -7874,13 +7874,13 @@
         <v>714</v>
       </c>
       <c r="O81">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="P81">
         <v>1</v>
       </c>
       <c r="Q81" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R81" t="s">
         <v>721</v>
@@ -7939,13 +7939,13 @@
         <v>716</v>
       </c>
       <c r="O82">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="P82">
         <v>1</v>
       </c>
       <c r="Q82" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R82" t="s">
         <v>721</v>
@@ -8004,7 +8004,7 @@
         <v>717</v>
       </c>
       <c r="O83">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="P83">
         <v>0</v>
@@ -8069,13 +8069,13 @@
         <v>716</v>
       </c>
       <c r="O84">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="P84">
         <v>2</v>
       </c>
       <c r="Q84" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R84" t="s">
         <v>721</v>
@@ -8134,7 +8134,7 @@
         <v>698</v>
       </c>
       <c r="O85">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="P85">
         <v>4</v>
@@ -8199,13 +8199,13 @@
         <v>698</v>
       </c>
       <c r="O86">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="P86">
         <v>1</v>
       </c>
       <c r="Q86" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R86" t="s">
         <v>721</v>
@@ -8264,7 +8264,7 @@
         <v>694</v>
       </c>
       <c r="O87">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="P87">
         <v>4</v>
@@ -8329,7 +8329,7 @@
         <v>691</v>
       </c>
       <c r="O88">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="P88">
         <v>0</v>
@@ -8394,7 +8394,7 @@
         <v>707</v>
       </c>
       <c r="O89">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="P89">
         <v>0</v>
@@ -8459,7 +8459,7 @@
         <v>692</v>
       </c>
       <c r="O90">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="P90">
         <v>0</v>
@@ -8524,7 +8524,7 @@
         <v>702</v>
       </c>
       <c r="O91">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="P91">
         <v>0</v>
@@ -8589,7 +8589,7 @@
         <v>710</v>
       </c>
       <c r="O92">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="P92">
         <v>0</v>
@@ -8654,7 +8654,7 @@
         <v>697</v>
       </c>
       <c r="O93">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="P93">
         <v>0</v>
@@ -8719,13 +8719,13 @@
         <v>703</v>
       </c>
       <c r="O94">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="P94">
         <v>1</v>
       </c>
       <c r="Q94" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R94" t="s">
         <v>721</v>
@@ -8784,7 +8784,7 @@
         <v>691</v>
       </c>
       <c r="O95">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="P95">
         <v>0</v>
@@ -8849,13 +8849,13 @@
         <v>710</v>
       </c>
       <c r="O96">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="P96">
         <v>2</v>
       </c>
       <c r="Q96" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R96" t="s">
         <v>721</v>
@@ -8914,7 +8914,7 @@
         <v>711</v>
       </c>
       <c r="O97">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="P97">
         <v>0</v>
@@ -8979,13 +8979,13 @@
         <v>696</v>
       </c>
       <c r="O98">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="P98">
         <v>1</v>
       </c>
       <c r="Q98" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R98" t="s">
         <v>721</v>
@@ -9044,7 +9044,7 @@
         <v>713</v>
       </c>
       <c r="O99">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="P99">
         <v>0</v>
@@ -9109,7 +9109,7 @@
         <v>706</v>
       </c>
       <c r="O100">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="P100">
         <v>0</v>
@@ -9174,13 +9174,13 @@
         <v>708</v>
       </c>
       <c r="O101">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="P101">
         <v>1</v>
       </c>
       <c r="Q101" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="R101" t="s">
         <v>721</v>

</xml_diff>